<commit_message>
Rename output sheet to Articles
</commit_message>
<xml_diff>
--- a/examples/turkish_politics_articles_database.sample.xlsx
+++ b/examples/turkish_politics_articles_database.sample.xlsx
@@ -6,11 +6,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Turkish Politics Articles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Articles" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Journal Directory" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Turkish Politics Articles'!$A$1:$I$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Articles'!$A$1:$I$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Journal Directory'!$A$1:$F$21</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Add added-at tracking and live sync progress
</commit_message>
<xml_diff>
--- a/examples/turkish_politics_articles_database.sample.xlsx
+++ b/examples/turkish_politics_articles_database.sample.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Articles" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Journal Directory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_openalex_sync_meta" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Articles'!$A$1:$I$46</definedName>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -477,6 +478,7 @@
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +527,11 @@
           <t>Key Topics</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Added At</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -570,6 +577,7 @@
           <t>Existing Topic, Demo Politics</t>
         </is>
       </c>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -615,6 +623,7 @@
           <t>Sample Topic, Public Demo</t>
         </is>
       </c>
+      <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1"/>
     <row r="5" ht="28" customHeight="1"/>
@@ -6712,4 +6721,40 @@
   <autoFilter ref="A1:F21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>work_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normalized_key</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>synced_at</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Split DOI and article URL with Crossref fallback
</commit_message>
<xml_diff>
--- a/examples/turkish_politics_articles_database.sample.xlsx
+++ b/examples/turkish_politics_articles_database.sample.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
@@ -514,20 +514,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>DOI/Link</t>
+          <t>DOI</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Article URL</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Cluster</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Key Topics</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Added At</t>
         </is>
@@ -567,17 +572,18 @@
           <t>https://doi.org/10.5555/sample-existing</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Turkey-dedicated</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Existing Topic, Demo Politics</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -608,22 +614,23 @@
           <t>33-47</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>https://example.org/sample-note</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Turkey-dedicated</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Sample Topic, Public Demo</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1"/>
     <row r="5" ht="28" customHeight="1"/>
@@ -6022,7 +6029,7 @@
   <autoFilter ref="A1:I46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add workbook settings and journal discovery workflow
</commit_message>
<xml_diff>
--- a/examples/turkish_politics_articles_database.sample.xlsx
+++ b/examples/turkish_politics_articles_database.sample.xlsx
@@ -8,7 +8,8 @@
   <sheets>
     <sheet name="Articles" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Journal Directory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="_openalex_sync_meta" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="Tracker Settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="_openalex_sync_meta" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Articles'!$A$1:$I$46</definedName>
@@ -6041,7 +6042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6050,6 +6051,7 @@
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6083,6 +6085,11 @@
           <t>Website</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Track?</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -6115,6 +6122,11 @@
           <t>https://www.tandfonline.com/journals/ftur20</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -6147,6 +6159,11 @@
           <t>https://www.cambridge.org/core/journals/new-perspectives-on-turkey</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -6179,6 +6196,11 @@
           <t>https://www.journalofdemocracy.org</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -6211,6 +6233,11 @@
           <t>https://www.tandfonline.com/journals/fdem20</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -6243,6 +6270,11 @@
           <t>https://www.cambridge.org/core/journals/government-and-opposition</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6275,6 +6307,11 @@
           <t>https://journals.sagepub.com/home/cps</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -6307,6 +6344,11 @@
           <t>https://journals.sagepub.com/home/ppq</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -6339,6 +6381,11 @@
           <t>https://www.cambridge.org/core/journals/international-journal-of-middle-east-studies</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -6371,6 +6418,11 @@
           <t>https://www.tandfonline.com/journals/fses20</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -6403,6 +6455,11 @@
           <t>https://www.tandfonline.com/journals/fmed20</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -6435,6 +6492,11 @@
           <t>https://www.tandfonline.com/journals/fmes20</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6467,6 +6529,11 @@
           <t>https://www.tandfonline.com/journals/fses20</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -6499,6 +6566,11 @@
           <t>https://www.tandfonline.com/journals/cbjm20</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6531,6 +6603,11 @@
           <t>https://www.tandfonline.com/journals/ctwq20</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6563,6 +6640,11 @@
           <t>https://onlinelibrary.wiley.com/journal/1467923x</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6595,6 +6677,11 @@
           <t>https://journals.sagepub.com/home/ann</t>
         </is>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6627,6 +6714,11 @@
           <t>https://www.cambridge.org/core/journals/world-politics</t>
         </is>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6659,6 +6751,11 @@
           <t>https://ejpr.onlinelibrary.wiley.com</t>
         </is>
       </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6691,6 +6788,11 @@
           <t>https://onlinelibrary.wiley.com/journal/14698129</t>
         </is>
       </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6721,6 +6823,11 @@
       <c r="F21" s="2" t="inlineStr">
         <is>
           <t>https://www.tandfonline.com/journals/rers20</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -6736,6 +6843,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Profile Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Workbook Starter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Articles Sheet</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Articles</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Journal Directory Sheet</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Journal Directory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>CSV Output</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Use Tracked Journals Only</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Crossref Mailto</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>